<commit_message>
added data to cherokee template
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee Freedman Minor.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee Freedman Minor.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -86,6 +86,12 @@
   </si>
   <si>
     <t>Image Binary</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Died prior to March 4, 1906; not entitled to land or money.</t>
   </si>
 </sst>
 </file>
@@ -9323,8 +9329,35 @@
         <f t="shared" si="20"/>
         <v>501</v>
       </c>
+      <c r="D444" t="s">
+        <v>25</v>
+      </c>
+      <c r="E444" t="s">
+        <v>24</v>
+      </c>
+      <c r="F444" t="s">
+        <v>24</v>
+      </c>
+      <c r="G444" t="s">
+        <v>24</v>
+      </c>
+      <c r="H444">
+        <v>-1</v>
+      </c>
+      <c r="I444" t="s">
+        <v>24</v>
+      </c>
+      <c r="J444" t="s">
+        <v>24</v>
+      </c>
+      <c r="K444" t="s">
+        <v>24</v>
+      </c>
       <c r="L444" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="M444" t="s">
+        <v>24</v>
       </c>
       <c r="N444" t="str">
         <f t="shared" si="21"/>
@@ -12481,8 +12514,35 @@
         <f t="shared" si="29"/>
         <v>502</v>
       </c>
+      <c r="D602" t="s">
+        <v>25</v>
+      </c>
+      <c r="E602" t="s">
+        <v>24</v>
+      </c>
+      <c r="F602" t="s">
+        <v>24</v>
+      </c>
+      <c r="G602" t="s">
+        <v>24</v>
+      </c>
+      <c r="H602">
+        <v>-1</v>
+      </c>
+      <c r="I602" t="s">
+        <v>24</v>
+      </c>
+      <c r="J602" t="s">
+        <v>24</v>
+      </c>
+      <c r="K602" t="s">
+        <v>24</v>
+      </c>
       <c r="L602" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="M602" t="s">
+        <v>24</v>
       </c>
       <c r="N602" t="str">
         <f t="shared" si="30"/>

</xml_diff>